<commit_message>
created an RTM using the web apps provided test cases. Added 7 more test cases to repository from the RTM
</commit_message>
<xml_diff>
--- a/Automation Exercise Project/Bug Report/Automation Exercise Defect Log.xlsx
+++ b/Automation Exercise Project/Bug Report/Automation Exercise Defect Log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kgmcm\OneDrive\Desktop\QA Portfolio\Qa-Portfolio\Bug Report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kgmcm\OneDrive\Desktop\QA Portfolio\Qa-Portfolio\Automation Exercise Project\Bug Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F86EDEA3-F114-4090-8194-970EA094FDC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E49824EF-021B-4340-A36B-309A3C7C123B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5130" yWindow="2970" windowWidth="28800" windowHeight="15370" xr2:uid="{950A3755-BD06-4699-808C-29ABC2B08016}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{950A3755-BD06-4699-808C-29ABC2B08016}"/>
   </bookViews>
   <sheets>
     <sheet name="Bug Report" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="71">
   <si>
     <t>Project: Automation Exercise Ecommerce Website QA Testing | Record one independently reproducible defect per row</t>
   </si>
@@ -135,11 +135,6 @@
   </si>
   <si>
     <t>High</t>
-  </si>
-  <si>
-    <t>Web application
-Browser/OS: Record during execution
-URL: https://automationexercise.com</t>
   </si>
   <si>
     <t>1. Active registered test account exists.
@@ -163,9 +158,6 @@
     <t>After logout, clicking the browser Back button displayed the previous page with “Logged in as Kevin Tester” and the Logout option. Further verification is required to determine whether the page was cached or the authenticated session remained active.</t>
   </si>
   <si>
-    <t>Add a redacted screenshot showing the stale authenticated interface.</t>
-  </si>
-  <si>
     <t>Not Retested</t>
   </si>
   <si>
@@ -176,12 +168,6 @@
   </si>
   <si>
     <t>Repeated logout request causes an unhandled KeyError and exposes internal debugging information</t>
-  </si>
-  <si>
-    <t>Web application
-Django 3.2.8 shown in response
-Python 3.7.17 shown in response
-URL: https://automationexercise.com/logout</t>
   </si>
   <si>
     <t>1. Open Automation Exercise.
@@ -199,12 +185,6 @@
     <t>The application displayed “KeyError at /logout” because the user_id session key was missing. A Django debug page exposed framework and Python versions, server paths, traceback details, cookies, and session-related information.</t>
   </si>
   <si>
-    <t>Add only a sanitized screenshot. Redact all cookie, session, username, token, and path values.</t>
-  </si>
-  <si>
-    <t>Security-relevant information disclosure. The original screenshot must not be published without extensive redaction.</t>
-  </si>
-  <si>
     <t>Automation Exercise Defect Reports</t>
   </si>
   <si>
@@ -218,6 +198,97 @@
   </si>
   <si>
     <t>Potential cached page behavior. Confirm session state by refreshing and accessing a protected feature before final severity assessment.</t>
+  </si>
+  <si>
+    <t>AE-BUG-003</t>
+  </si>
+  <si>
+    <t>AE-CART-001</t>
+  </si>
+  <si>
+    <t>Cart</t>
+  </si>
+  <si>
+    <t>Functional / Calculation Display</t>
+  </si>
+  <si>
+    <t>Cart does not display the overall total after multiple products are added</t>
+  </si>
+  <si>
+    <t>Web application
+Brave v193.129/Win11
+URL: https://automationexercise.com</t>
+  </si>
+  <si>
+    <t>Web application
+Brave v193.129/Win11
+Django 3.2.8 shown in response
+Python 3.7.17 shown in response
+URL: https://automationexercise.com/logout</t>
+  </si>
+  <si>
+    <t>Web application
+Brave v193.129/Win11</t>
+  </si>
+  <si>
+    <t>1. Website is available
+2. User is logged out
+3. At least two products are available</t>
+  </si>
+  <si>
+    <t>1. Open https://automationexercise.com while logged out.
+2. Click the Products button.
+3. Add the first product to the cart.
+4. Click Continue Shopping.
+5. Add the second product to the cart.
+6. Click View Cart.
+7. Verify that both products appear in the cart.
+8. Review the prices, quantities, line totals, and overall cart total.</t>
+  </si>
+  <si>
+    <t>Both products should appear with the correct unit prices, quantities, and line totals. The cart should also display an accurate overall total equal to the sum of all product line totals.</t>
+  </si>
+  <si>
+    <t>Both products appear with the correct unit prices, quantities, and line totals, but the overall cart total is not displayed.</t>
+  </si>
+  <si>
+    <t>..\Screenshots\AE-LOGOUT-001.png</t>
+  </si>
+  <si>
+    <t>..\Screenshots\AE-CART-001.png</t>
+  </si>
+  <si>
+    <t>Meta data, session tokens and cookies blurred in screenshot</t>
+  </si>
+  <si>
+    <t>AE-BUG-004</t>
+  </si>
+  <si>
+    <t>AE-CART-002</t>
+  </si>
+  <si>
+    <t>Functional / User Interface</t>
+  </si>
+  <si>
+    <t>The quantity field on the product-detail page does not respond when the user attempts to edit it. As a result, the user cannot select the desired quantity before adding the product to the cart.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open https://automationexercise.com while logged out.
+2. Click View Product for any available product.
+3. Add product to Cart
+4. View Cart
+5. Click inside the quantity field.
+6. Attempt to change the quantity from 1 to 4.
+</t>
+  </si>
+  <si>
+    <t>The quantity field should accept a valid quantity of 4. After the product is added, the cart should display the selected product with a quantity of 4 and a line total equal to the unit price multiplied by 4</t>
+  </si>
+  <si>
+    <t>..\Screenshots\AE-CART-002.png</t>
+  </si>
+  <si>
+    <t>The populated cart page is displayed, but the quantity field cannot be edited. Clicking the field produces no response, preventing the user from selecting a quantity of 4.</t>
   </si>
 </sst>
 </file>
@@ -227,7 +298,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -276,6 +347,14 @@
       <color rgb="FF1F2937"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -310,7 +389,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -439,48 +518,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -503,8 +560,51 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="9">
@@ -992,841 +1092,909 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="34" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
+      <c r="A1" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="11"/>
+      <c r="Q1" s="11"/>
+      <c r="R1" s="11"/>
+      <c r="S1" s="11"/>
+      <c r="T1" s="11"/>
+      <c r="U1" s="11"/>
     </row>
     <row r="2" spans="1:21" ht="23" customHeight="1">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="2"/>
-      <c r="S2" s="2"/>
-      <c r="T2" s="2"/>
-      <c r="U2" s="2"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12"/>
+      <c r="T2" s="12"/>
+      <c r="U2" s="12"/>
     </row>
     <row r="4" spans="1:21">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="D4" s="3" t="s">
+      <c r="B4" s="14"/>
+      <c r="D4" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="G4" s="3" t="s">
+      <c r="E4" s="14"/>
+      <c r="G4" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="4"/>
-      <c r="J4" s="3" t="s">
+      <c r="H4" s="14"/>
+      <c r="J4" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="4"/>
-      <c r="M4" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="6"/>
-      <c r="T4" s="6"/>
-      <c r="U4" s="7"/>
+      <c r="K4" s="14"/>
+      <c r="M4" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="N4" s="16"/>
+      <c r="O4" s="16"/>
+      <c r="P4" s="16"/>
+      <c r="Q4" s="16"/>
+      <c r="R4" s="16"/>
+      <c r="S4" s="16"/>
+      <c r="T4" s="16"/>
+      <c r="U4" s="17"/>
     </row>
     <row r="5" spans="1:21" ht="19">
-      <c r="A5" s="8">
+      <c r="A5" s="9">
         <f>COUNTA(A8:A107)</f>
+        <v>4</v>
+      </c>
+      <c r="B5" s="10"/>
+      <c r="D5" s="9">
+        <f>COUNTIF(M8:M107,"Open")</f>
+        <v>4</v>
+      </c>
+      <c r="E5" s="10"/>
+      <c r="G5" s="9">
+        <f>COUNTIF(F8:F107,"High")+COUNTIF(F8:F107,"Critical")</f>
         <v>2</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="D5" s="8">
-        <f>COUNTIF(M8:M107,"Open")</f>
-        <v>2</v>
-      </c>
-      <c r="E5" s="9"/>
-      <c r="G5" s="8">
-        <f>COUNTIF(F8:F107,"High")+COUNTIF(F8:F107,"Critical")</f>
-        <v>1</v>
-      </c>
-      <c r="H5" s="9"/>
-      <c r="J5" s="8">
+      <c r="H5" s="10"/>
+      <c r="J5" s="9">
         <f>COUNTIF(M8:M107,"Ready for Retest")</f>
         <v>0</v>
       </c>
-      <c r="K5" s="9"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="11"/>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="11"/>
-      <c r="R5" s="11"/>
-      <c r="S5" s="11"/>
-      <c r="T5" s="11"/>
-      <c r="U5" s="12"/>
+      <c r="K5" s="10"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="19"/>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="19"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="19"/>
+      <c r="U5" s="20"/>
     </row>
     <row r="7" spans="1:21" ht="40" customHeight="1">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="O7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="P7" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="R7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="S7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="T7" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="U7" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" ht="130.5" customHeight="1">
+      <c r="A8" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="M8" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="N8" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="O8" s="8">
+        <v>46232</v>
+      </c>
+      <c r="P8" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q8" s="6"/>
+      <c r="R8" s="6"/>
+      <c r="S8" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="T8" s="8"/>
+      <c r="U8" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" ht="93.5" customHeight="1">
+      <c r="A9" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="M9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="N9" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="O9" s="8">
+        <v>46232</v>
+      </c>
+      <c r="P9" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="6"/>
+      <c r="S9" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="T9" s="8"/>
+      <c r="U9" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" ht="126" customHeight="1">
+      <c r="A10" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="G7" s="17" t="s">
-        <v>10</v>
-      </c>
-      <c r="H7" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="I7" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="J7" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="K7" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="L7" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="M7" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="N7" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="O7" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="P7" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q7" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R7" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="S7" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="T7" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="U7" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" ht="130.5" customHeight="1">
-      <c r="A8" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="E8" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="F8" s="18" t="s">
+      <c r="C10" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="F10" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="G10" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="H8" s="19" t="s">
-        <v>32</v>
-      </c>
-      <c r="I8" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="J8" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="K8" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="L8" s="19" t="s">
+      <c r="H10" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="M10" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="N10" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="O10" s="8">
+        <v>46233</v>
+      </c>
+      <c r="P10" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q10" s="6"/>
+      <c r="R10" s="6"/>
+      <c r="S10" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="M8" s="18" t="s">
+      <c r="T10" s="8"/>
+      <c r="U10" s="6"/>
+    </row>
+    <row r="11" spans="1:21" ht="87" customHeight="1">
+      <c r="A11" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="M11" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="N8" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="O8" s="20">
-        <v>46232</v>
-      </c>
-      <c r="P8" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q8" s="18"/>
-      <c r="R8" s="18"/>
-      <c r="S8" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="T8" s="20"/>
-      <c r="U8" s="18" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" ht="93.5" customHeight="1">
-      <c r="A9" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="E9" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="G9" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="H9" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="I9" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="J9" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="K9" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="L9" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="M9" s="18" t="s">
-        <v>2</v>
-      </c>
-      <c r="N9" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="O9" s="20">
-        <v>46232</v>
-      </c>
-      <c r="P9" s="18" t="s">
+      <c r="N11" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="Q9" s="18"/>
-      <c r="R9" s="18"/>
-      <c r="S9" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="T9" s="20"/>
-      <c r="U9" s="18" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" ht="42" customHeight="1">
-      <c r="A10" s="18"/>
-      <c r="B10" s="18"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
-      <c r="L10" s="19"/>
-      <c r="M10" s="18"/>
-      <c r="N10" s="18"/>
-      <c r="O10" s="20"/>
-      <c r="P10" s="18"/>
-      <c r="Q10" s="18"/>
-      <c r="R10" s="18"/>
-      <c r="S10" s="18"/>
-      <c r="T10" s="20"/>
-      <c r="U10" s="18"/>
-    </row>
-    <row r="11" spans="1:21" ht="42" customHeight="1">
-      <c r="A11" s="18"/>
-      <c r="B11" s="18"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="19"/>
-      <c r="K11" s="19"/>
-      <c r="L11" s="19"/>
-      <c r="M11" s="18"/>
-      <c r="N11" s="18"/>
-      <c r="O11" s="20"/>
-      <c r="P11" s="18"/>
-      <c r="Q11" s="18"/>
-      <c r="R11" s="18"/>
-      <c r="S11" s="18"/>
-      <c r="T11" s="20"/>
-      <c r="U11" s="18"/>
+      <c r="O11" s="8">
+        <v>46234</v>
+      </c>
+      <c r="P11" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q11" s="6"/>
+      <c r="R11" s="6"/>
+      <c r="S11" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="T11" s="8"/>
+      <c r="U11" s="6"/>
     </row>
     <row r="12" spans="1:21" ht="42" customHeight="1">
-      <c r="A12" s="18"/>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="19"/>
-      <c r="I12" s="19"/>
-      <c r="J12" s="19"/>
-      <c r="K12" s="19"/>
-      <c r="L12" s="19"/>
-      <c r="M12" s="18"/>
-      <c r="N12" s="18"/>
-      <c r="O12" s="20"/>
-      <c r="P12" s="18"/>
-      <c r="Q12" s="18"/>
-      <c r="R12" s="18"/>
-      <c r="S12" s="18"/>
-      <c r="T12" s="20"/>
-      <c r="U12" s="18"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="6"/>
+      <c r="Q12" s="6"/>
+      <c r="R12" s="6"/>
+      <c r="S12" s="6"/>
+      <c r="T12" s="8"/>
+      <c r="U12" s="6"/>
     </row>
     <row r="13" spans="1:21" ht="42" customHeight="1">
-      <c r="A13" s="18"/>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="19"/>
-      <c r="J13" s="19"/>
-      <c r="K13" s="19"/>
-      <c r="L13" s="19"/>
-      <c r="M13" s="18"/>
-      <c r="N13" s="18"/>
-      <c r="O13" s="20"/>
-      <c r="P13" s="18"/>
-      <c r="Q13" s="18"/>
-      <c r="R13" s="18"/>
-      <c r="S13" s="18"/>
-      <c r="T13" s="20"/>
-      <c r="U13" s="18"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6"/>
+      <c r="S13" s="6"/>
+      <c r="T13" s="8"/>
+      <c r="U13" s="6"/>
     </row>
     <row r="14" spans="1:21" ht="42" customHeight="1">
-      <c r="A14" s="18"/>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="19"/>
-      <c r="I14" s="19"/>
-      <c r="J14" s="19"/>
-      <c r="K14" s="19"/>
-      <c r="L14" s="19"/>
-      <c r="M14" s="18"/>
-      <c r="N14" s="18"/>
-      <c r="O14" s="20"/>
-      <c r="P14" s="18"/>
-      <c r="Q14" s="18"/>
-      <c r="R14" s="18"/>
-      <c r="S14" s="18"/>
-      <c r="T14" s="20"/>
-      <c r="U14" s="18"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="6"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="6"/>
+      <c r="Q14" s="6"/>
+      <c r="R14" s="6"/>
+      <c r="S14" s="6"/>
+      <c r="T14" s="8"/>
+      <c r="U14" s="6"/>
     </row>
     <row r="15" spans="1:21" ht="42" customHeight="1">
-      <c r="A15" s="18"/>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="19"/>
-      <c r="J15" s="19"/>
-      <c r="K15" s="19"/>
-      <c r="L15" s="19"/>
-      <c r="M15" s="18"/>
-      <c r="N15" s="18"/>
-      <c r="O15" s="20"/>
-      <c r="P15" s="18"/>
-      <c r="Q15" s="18"/>
-      <c r="R15" s="18"/>
-      <c r="S15" s="18"/>
-      <c r="T15" s="20"/>
-      <c r="U15" s="18"/>
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="6"/>
+      <c r="N15" s="6"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="6"/>
+      <c r="Q15" s="6"/>
+      <c r="R15" s="6"/>
+      <c r="S15" s="6"/>
+      <c r="T15" s="8"/>
+      <c r="U15" s="6"/>
     </row>
     <row r="16" spans="1:21" ht="42" customHeight="1">
-      <c r="A16" s="18"/>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="19"/>
-      <c r="J16" s="19"/>
-      <c r="K16" s="19"/>
-      <c r="L16" s="19"/>
-      <c r="M16" s="18"/>
-      <c r="N16" s="18"/>
-      <c r="O16" s="20"/>
-      <c r="P16" s="18"/>
-      <c r="Q16" s="18"/>
-      <c r="R16" s="18"/>
-      <c r="S16" s="18"/>
-      <c r="T16" s="20"/>
-      <c r="U16" s="18"/>
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="7"/>
+      <c r="K16" s="7"/>
+      <c r="L16" s="7"/>
+      <c r="M16" s="6"/>
+      <c r="N16" s="6"/>
+      <c r="O16" s="8"/>
+      <c r="P16" s="6"/>
+      <c r="Q16" s="6"/>
+      <c r="R16" s="6"/>
+      <c r="S16" s="6"/>
+      <c r="T16" s="8"/>
+      <c r="U16" s="6"/>
     </row>
     <row r="17" spans="1:21" ht="42" customHeight="1">
-      <c r="A17" s="13"/>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="14"/>
-      <c r="L17" s="14"/>
-      <c r="M17" s="13"/>
-      <c r="N17" s="13"/>
-      <c r="O17" s="15"/>
-      <c r="P17" s="13"/>
-      <c r="Q17" s="13"/>
-      <c r="R17" s="13"/>
-      <c r="S17" s="13"/>
-      <c r="T17" s="15"/>
-      <c r="U17" s="13"/>
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+      <c r="L17" s="2"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="3"/>
+      <c r="P17" s="1"/>
+      <c r="Q17" s="1"/>
+      <c r="R17" s="1"/>
+      <c r="S17" s="1"/>
+      <c r="T17" s="3"/>
+      <c r="U17" s="1"/>
     </row>
     <row r="18" spans="1:21">
-      <c r="O18" s="16"/>
-      <c r="T18" s="16"/>
+      <c r="O18" s="4"/>
+      <c r="T18" s="4"/>
     </row>
     <row r="19" spans="1:21">
-      <c r="O19" s="16"/>
-      <c r="T19" s="16"/>
+      <c r="O19" s="4"/>
+      <c r="T19" s="4"/>
     </row>
     <row r="20" spans="1:21">
-      <c r="O20" s="16"/>
-      <c r="T20" s="16"/>
+      <c r="O20" s="4"/>
+      <c r="T20" s="4"/>
     </row>
     <row r="21" spans="1:21">
-      <c r="O21" s="16"/>
-      <c r="T21" s="16"/>
+      <c r="O21" s="4"/>
+      <c r="T21" s="4"/>
     </row>
     <row r="22" spans="1:21">
-      <c r="O22" s="16"/>
-      <c r="T22" s="16"/>
+      <c r="O22" s="4"/>
+      <c r="T22" s="4"/>
     </row>
     <row r="23" spans="1:21">
-      <c r="O23" s="16"/>
-      <c r="T23" s="16"/>
+      <c r="O23" s="4"/>
+      <c r="T23" s="4"/>
     </row>
     <row r="24" spans="1:21">
-      <c r="O24" s="16"/>
-      <c r="T24" s="16"/>
+      <c r="O24" s="4"/>
+      <c r="T24" s="4"/>
     </row>
     <row r="25" spans="1:21">
-      <c r="O25" s="16"/>
-      <c r="T25" s="16"/>
+      <c r="O25" s="4"/>
+      <c r="T25" s="4"/>
     </row>
     <row r="26" spans="1:21">
-      <c r="O26" s="16"/>
-      <c r="T26" s="16"/>
+      <c r="O26" s="4"/>
+      <c r="T26" s="4"/>
     </row>
     <row r="27" spans="1:21">
-      <c r="O27" s="16"/>
-      <c r="T27" s="16"/>
+      <c r="O27" s="4"/>
+      <c r="T27" s="4"/>
     </row>
     <row r="28" spans="1:21">
-      <c r="O28" s="16"/>
-      <c r="T28" s="16"/>
+      <c r="O28" s="4"/>
+      <c r="T28" s="4"/>
     </row>
     <row r="29" spans="1:21">
-      <c r="O29" s="16"/>
-      <c r="T29" s="16"/>
+      <c r="O29" s="4"/>
+      <c r="T29" s="4"/>
     </row>
     <row r="30" spans="1:21">
-      <c r="O30" s="16"/>
-      <c r="T30" s="16"/>
+      <c r="O30" s="4"/>
+      <c r="T30" s="4"/>
     </row>
     <row r="31" spans="1:21">
-      <c r="O31" s="16"/>
-      <c r="T31" s="16"/>
+      <c r="O31" s="4"/>
+      <c r="T31" s="4"/>
     </row>
     <row r="32" spans="1:21">
-      <c r="O32" s="16"/>
-      <c r="T32" s="16"/>
+      <c r="O32" s="4"/>
+      <c r="T32" s="4"/>
     </row>
     <row r="33" spans="15:20">
-      <c r="O33" s="16"/>
-      <c r="T33" s="16"/>
+      <c r="O33" s="4"/>
+      <c r="T33" s="4"/>
     </row>
     <row r="34" spans="15:20">
-      <c r="O34" s="16"/>
-      <c r="T34" s="16"/>
+      <c r="O34" s="4"/>
+      <c r="T34" s="4"/>
     </row>
     <row r="35" spans="15:20">
-      <c r="O35" s="16"/>
-      <c r="T35" s="16"/>
+      <c r="O35" s="4"/>
+      <c r="T35" s="4"/>
     </row>
     <row r="36" spans="15:20">
-      <c r="O36" s="16"/>
-      <c r="T36" s="16"/>
+      <c r="O36" s="4"/>
+      <c r="T36" s="4"/>
     </row>
     <row r="37" spans="15:20">
-      <c r="O37" s="16"/>
-      <c r="T37" s="16"/>
+      <c r="O37" s="4"/>
+      <c r="T37" s="4"/>
     </row>
     <row r="38" spans="15:20">
-      <c r="O38" s="16"/>
-      <c r="T38" s="16"/>
+      <c r="O38" s="4"/>
+      <c r="T38" s="4"/>
     </row>
     <row r="39" spans="15:20">
-      <c r="O39" s="16"/>
-      <c r="T39" s="16"/>
+      <c r="O39" s="4"/>
+      <c r="T39" s="4"/>
     </row>
     <row r="40" spans="15:20">
-      <c r="O40" s="16"/>
-      <c r="T40" s="16"/>
+      <c r="O40" s="4"/>
+      <c r="T40" s="4"/>
     </row>
     <row r="41" spans="15:20">
-      <c r="O41" s="16"/>
-      <c r="T41" s="16"/>
+      <c r="O41" s="4"/>
+      <c r="T41" s="4"/>
     </row>
     <row r="42" spans="15:20">
-      <c r="O42" s="16"/>
-      <c r="T42" s="16"/>
+      <c r="O42" s="4"/>
+      <c r="T42" s="4"/>
     </row>
     <row r="43" spans="15:20">
-      <c r="O43" s="16"/>
-      <c r="T43" s="16"/>
+      <c r="O43" s="4"/>
+      <c r="T43" s="4"/>
     </row>
     <row r="44" spans="15:20">
-      <c r="O44" s="16"/>
-      <c r="T44" s="16"/>
+      <c r="O44" s="4"/>
+      <c r="T44" s="4"/>
     </row>
     <row r="45" spans="15:20">
-      <c r="O45" s="16"/>
-      <c r="T45" s="16"/>
+      <c r="O45" s="4"/>
+      <c r="T45" s="4"/>
     </row>
     <row r="46" spans="15:20">
-      <c r="O46" s="16"/>
-      <c r="T46" s="16"/>
+      <c r="O46" s="4"/>
+      <c r="T46" s="4"/>
     </row>
     <row r="47" spans="15:20">
-      <c r="O47" s="16"/>
-      <c r="T47" s="16"/>
+      <c r="O47" s="4"/>
+      <c r="T47" s="4"/>
     </row>
     <row r="48" spans="15:20">
-      <c r="O48" s="16"/>
-      <c r="T48" s="16"/>
+      <c r="O48" s="4"/>
+      <c r="T48" s="4"/>
     </row>
     <row r="49" spans="15:20">
-      <c r="O49" s="16"/>
-      <c r="T49" s="16"/>
+      <c r="O49" s="4"/>
+      <c r="T49" s="4"/>
     </row>
     <row r="50" spans="15:20">
-      <c r="O50" s="16"/>
-      <c r="T50" s="16"/>
+      <c r="O50" s="4"/>
+      <c r="T50" s="4"/>
     </row>
     <row r="51" spans="15:20">
-      <c r="O51" s="16"/>
-      <c r="T51" s="16"/>
+      <c r="O51" s="4"/>
+      <c r="T51" s="4"/>
     </row>
     <row r="52" spans="15:20">
-      <c r="O52" s="16"/>
-      <c r="T52" s="16"/>
+      <c r="O52" s="4"/>
+      <c r="T52" s="4"/>
     </row>
     <row r="53" spans="15:20">
-      <c r="O53" s="16"/>
-      <c r="T53" s="16"/>
+      <c r="O53" s="4"/>
+      <c r="T53" s="4"/>
     </row>
     <row r="54" spans="15:20">
-      <c r="O54" s="16"/>
-      <c r="T54" s="16"/>
+      <c r="O54" s="4"/>
+      <c r="T54" s="4"/>
     </row>
     <row r="55" spans="15:20">
-      <c r="O55" s="16"/>
-      <c r="T55" s="16"/>
+      <c r="O55" s="4"/>
+      <c r="T55" s="4"/>
     </row>
     <row r="56" spans="15:20">
-      <c r="O56" s="16"/>
-      <c r="T56" s="16"/>
+      <c r="O56" s="4"/>
+      <c r="T56" s="4"/>
     </row>
     <row r="57" spans="15:20">
-      <c r="O57" s="16"/>
-      <c r="T57" s="16"/>
+      <c r="O57" s="4"/>
+      <c r="T57" s="4"/>
     </row>
     <row r="58" spans="15:20">
-      <c r="O58" s="16"/>
-      <c r="T58" s="16"/>
+      <c r="O58" s="4"/>
+      <c r="T58" s="4"/>
     </row>
     <row r="59" spans="15:20">
-      <c r="O59" s="16"/>
-      <c r="T59" s="16"/>
+      <c r="O59" s="4"/>
+      <c r="T59" s="4"/>
     </row>
     <row r="60" spans="15:20">
-      <c r="O60" s="16"/>
-      <c r="T60" s="16"/>
+      <c r="O60" s="4"/>
+      <c r="T60" s="4"/>
     </row>
     <row r="61" spans="15:20">
-      <c r="O61" s="16"/>
-      <c r="T61" s="16"/>
+      <c r="O61" s="4"/>
+      <c r="T61" s="4"/>
     </row>
     <row r="62" spans="15:20">
-      <c r="O62" s="16"/>
-      <c r="T62" s="16"/>
+      <c r="O62" s="4"/>
+      <c r="T62" s="4"/>
     </row>
     <row r="63" spans="15:20">
-      <c r="O63" s="16"/>
-      <c r="T63" s="16"/>
+      <c r="O63" s="4"/>
+      <c r="T63" s="4"/>
     </row>
     <row r="64" spans="15:20">
-      <c r="O64" s="16"/>
-      <c r="T64" s="16"/>
+      <c r="O64" s="4"/>
+      <c r="T64" s="4"/>
     </row>
     <row r="65" spans="15:20">
-      <c r="O65" s="16"/>
-      <c r="T65" s="16"/>
+      <c r="O65" s="4"/>
+      <c r="T65" s="4"/>
     </row>
     <row r="66" spans="15:20">
-      <c r="O66" s="16"/>
-      <c r="T66" s="16"/>
+      <c r="O66" s="4"/>
+      <c r="T66" s="4"/>
     </row>
     <row r="67" spans="15:20">
-      <c r="O67" s="16"/>
-      <c r="T67" s="16"/>
+      <c r="O67" s="4"/>
+      <c r="T67" s="4"/>
     </row>
     <row r="68" spans="15:20">
-      <c r="O68" s="16"/>
-      <c r="T68" s="16"/>
+      <c r="O68" s="4"/>
+      <c r="T68" s="4"/>
     </row>
     <row r="69" spans="15:20">
-      <c r="O69" s="16"/>
-      <c r="T69" s="16"/>
+      <c r="O69" s="4"/>
+      <c r="T69" s="4"/>
     </row>
     <row r="70" spans="15:20">
-      <c r="O70" s="16"/>
-      <c r="T70" s="16"/>
+      <c r="O70" s="4"/>
+      <c r="T70" s="4"/>
     </row>
     <row r="71" spans="15:20">
-      <c r="O71" s="16"/>
-      <c r="T71" s="16"/>
+      <c r="O71" s="4"/>
+      <c r="T71" s="4"/>
     </row>
     <row r="72" spans="15:20">
-      <c r="O72" s="16"/>
-      <c r="T72" s="16"/>
+      <c r="O72" s="4"/>
+      <c r="T72" s="4"/>
     </row>
     <row r="73" spans="15:20">
-      <c r="O73" s="16"/>
-      <c r="T73" s="16"/>
+      <c r="O73" s="4"/>
+      <c r="T73" s="4"/>
     </row>
     <row r="74" spans="15:20">
-      <c r="O74" s="16"/>
-      <c r="T74" s="16"/>
+      <c r="O74" s="4"/>
+      <c r="T74" s="4"/>
     </row>
     <row r="75" spans="15:20">
-      <c r="O75" s="16"/>
-      <c r="T75" s="16"/>
+      <c r="O75" s="4"/>
+      <c r="T75" s="4"/>
     </row>
     <row r="76" spans="15:20">
-      <c r="O76" s="16"/>
-      <c r="T76" s="16"/>
+      <c r="O76" s="4"/>
+      <c r="T76" s="4"/>
     </row>
     <row r="77" spans="15:20">
-      <c r="O77" s="16"/>
-      <c r="T77" s="16"/>
+      <c r="O77" s="4"/>
+      <c r="T77" s="4"/>
     </row>
     <row r="78" spans="15:20">
-      <c r="O78" s="16"/>
-      <c r="T78" s="16"/>
+      <c r="O78" s="4"/>
+      <c r="T78" s="4"/>
     </row>
     <row r="79" spans="15:20">
-      <c r="O79" s="16"/>
-      <c r="T79" s="16"/>
+      <c r="O79" s="4"/>
+      <c r="T79" s="4"/>
     </row>
     <row r="80" spans="15:20">
-      <c r="O80" s="16"/>
-      <c r="T80" s="16"/>
+      <c r="O80" s="4"/>
+      <c r="T80" s="4"/>
     </row>
     <row r="81" spans="15:20">
-      <c r="O81" s="16"/>
-      <c r="T81" s="16"/>
+      <c r="O81" s="4"/>
+      <c r="T81" s="4"/>
     </row>
     <row r="82" spans="15:20">
-      <c r="O82" s="16"/>
-      <c r="T82" s="16"/>
+      <c r="O82" s="4"/>
+      <c r="T82" s="4"/>
     </row>
     <row r="83" spans="15:20">
-      <c r="O83" s="16"/>
-      <c r="T83" s="16"/>
+      <c r="O83" s="4"/>
+      <c r="T83" s="4"/>
     </row>
     <row r="84" spans="15:20">
-      <c r="O84" s="16"/>
-      <c r="T84" s="16"/>
+      <c r="O84" s="4"/>
+      <c r="T84" s="4"/>
     </row>
     <row r="85" spans="15:20">
-      <c r="O85" s="16"/>
-      <c r="T85" s="16"/>
+      <c r="O85" s="4"/>
+      <c r="T85" s="4"/>
     </row>
     <row r="86" spans="15:20">
-      <c r="O86" s="16"/>
-      <c r="T86" s="16"/>
+      <c r="O86" s="4"/>
+      <c r="T86" s="4"/>
     </row>
     <row r="87" spans="15:20">
-      <c r="O87" s="16"/>
-      <c r="T87" s="16"/>
+      <c r="O87" s="4"/>
+      <c r="T87" s="4"/>
     </row>
     <row r="88" spans="15:20">
-      <c r="O88" s="16"/>
-      <c r="T88" s="16"/>
+      <c r="O88" s="4"/>
+      <c r="T88" s="4"/>
     </row>
     <row r="89" spans="15:20">
-      <c r="O89" s="16"/>
-      <c r="T89" s="16"/>
+      <c r="O89" s="4"/>
+      <c r="T89" s="4"/>
     </row>
     <row r="90" spans="15:20">
-      <c r="O90" s="16"/>
-      <c r="T90" s="16"/>
+      <c r="O90" s="4"/>
+      <c r="T90" s="4"/>
     </row>
     <row r="91" spans="15:20">
-      <c r="O91" s="16"/>
-      <c r="T91" s="16"/>
+      <c r="O91" s="4"/>
+      <c r="T91" s="4"/>
     </row>
     <row r="92" spans="15:20">
-      <c r="O92" s="16"/>
-      <c r="T92" s="16"/>
+      <c r="O92" s="4"/>
+      <c r="T92" s="4"/>
     </row>
     <row r="93" spans="15:20">
-      <c r="O93" s="16"/>
-      <c r="T93" s="16"/>
+      <c r="O93" s="4"/>
+      <c r="T93" s="4"/>
     </row>
     <row r="94" spans="15:20">
-      <c r="O94" s="16"/>
-      <c r="T94" s="16"/>
+      <c r="O94" s="4"/>
+      <c r="T94" s="4"/>
     </row>
     <row r="95" spans="15:20">
-      <c r="O95" s="16"/>
-      <c r="T95" s="16"/>
+      <c r="O95" s="4"/>
+      <c r="T95" s="4"/>
     </row>
     <row r="96" spans="15:20">
-      <c r="O96" s="16"/>
-      <c r="T96" s="16"/>
+      <c r="O96" s="4"/>
+      <c r="T96" s="4"/>
     </row>
     <row r="97" spans="15:20">
-      <c r="O97" s="16"/>
-      <c r="T97" s="16"/>
+      <c r="O97" s="4"/>
+      <c r="T97" s="4"/>
     </row>
     <row r="98" spans="15:20">
-      <c r="O98" s="16"/>
-      <c r="T98" s="16"/>
+      <c r="O98" s="4"/>
+      <c r="T98" s="4"/>
     </row>
     <row r="99" spans="15:20">
-      <c r="O99" s="16"/>
-      <c r="T99" s="16"/>
+      <c r="O99" s="4"/>
+      <c r="T99" s="4"/>
     </row>
     <row r="100" spans="15:20">
-      <c r="O100" s="16"/>
-      <c r="T100" s="16"/>
+      <c r="O100" s="4"/>
+      <c r="T100" s="4"/>
     </row>
     <row r="101" spans="15:20">
-      <c r="O101" s="16"/>
-      <c r="T101" s="16"/>
+      <c r="O101" s="4"/>
+      <c r="T101" s="4"/>
     </row>
     <row r="102" spans="15:20">
-      <c r="O102" s="16"/>
-      <c r="T102" s="16"/>
+      <c r="O102" s="4"/>
+      <c r="T102" s="4"/>
     </row>
     <row r="103" spans="15:20">
-      <c r="O103" s="16"/>
-      <c r="T103" s="16"/>
+      <c r="O103" s="4"/>
+      <c r="T103" s="4"/>
     </row>
     <row r="104" spans="15:20">
-      <c r="O104" s="16"/>
-      <c r="T104" s="16"/>
+      <c r="O104" s="4"/>
+      <c r="T104" s="4"/>
     </row>
     <row r="105" spans="15:20">
-      <c r="O105" s="16"/>
-      <c r="T105" s="16"/>
+      <c r="O105" s="4"/>
+      <c r="T105" s="4"/>
     </row>
     <row r="106" spans="15:20">
-      <c r="O106" s="16"/>
-      <c r="T106" s="16"/>
+      <c r="O106" s="4"/>
+      <c r="T106" s="4"/>
     </row>
     <row r="107" spans="15:20">
-      <c r="O107" s="16"/>
-      <c r="T107" s="16"/>
+      <c r="O107" s="4"/>
+      <c r="T107" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -1857,7 +2025,7 @@
     <cfRule type="containsText" dxfId="1" priority="8" operator="containsText" text="Fail"/>
     <cfRule type="containsText" dxfId="0" priority="9" operator="containsText" text="Not Retested"/>
   </conditionalFormatting>
-  <dataValidations count="5">
+  <dataValidations count="8">
     <dataValidation type="list" sqref="S8:S107" xr:uid="{285366EE-0383-4ECF-AF60-BFA7FE11B678}">
       <formula1>"Not Retested,Pass,Fail,Blocked"</formula1>
     </dataValidation>
@@ -1867,16 +2035,31 @@
     <dataValidation type="list" sqref="F8:G107" xr:uid="{9975D9DE-3FF0-49C3-8240-A0EDA31122CB}">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="D8:D107" xr:uid="{20609973-F954-420B-A272-D9DA30F7C1CD}">
+    <dataValidation type="list" sqref="D17:D107" xr:uid="{20609973-F954-420B-A272-D9DA30F7C1CD}">
       <formula1>"Functional,Validation,Session / Navigation,Error Handling,Security / Information Disclosure,Usability,Data Integrity,Performance"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="C8:C107" xr:uid="{009EC8DC-924F-45F0-8799-8E0DEEBB0305}">
+    <dataValidation type="list" sqref="C17:C107" xr:uid="{009EC8DC-924F-45F0-8799-8E0DEEBB0305}">
       <formula1>"Signup,Login,Logout,Account Management"</formula1>
     </dataValidation>
+    <dataValidation type="list" sqref="C8:C16" xr:uid="{2E7BF27D-A7D0-4C6A-9B5A-85311896C1AB}">
+      <formula1>"Signup,Login,Logout,Account Management,Cart,Product"</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="D8:D10 D12:D16" xr:uid="{7E090F43-EDD5-4B08-B8EA-B310B818ACBC}">
+      <formula1>"Functional,Validation,Session / Navigation,Error Handling,Security / Information Disclosure,Usability,Data Integrity,Performance, Functional / Calculation Display"</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="D11" xr:uid="{3ADA1B1F-1171-4E65-9279-D6B3FE66D1BA}">
+      <formula1>"Functional,Validation,Session / Navigation,Error Handling,Security / Information Disclosure,Usability,Data Integrity,Performance, Functional / Calculation Display, Functional / User Interface"</formula1>
+    </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="P8" r:id="rId1" xr:uid="{EF999C47-803A-403B-956C-B7516530B5D0}"/>
+    <hyperlink ref="P9" r:id="rId2" xr:uid="{17F25047-CB4F-4BAB-8DA4-BDC57C5E51D5}"/>
+    <hyperlink ref="P10" r:id="rId3" xr:uid="{5587106D-E68A-4850-8D5E-C61D8AB13A2F}"/>
+    <hyperlink ref="P11" r:id="rId4" xr:uid="{9938056D-DD42-4172-A4D0-D75E65A74177}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: complete portfolio closeout
</commit_message>
<xml_diff>
--- a/Automation Exercise Project/Bug Report/Automation Exercise Defect Log.xlsx
+++ b/Automation Exercise Project/Bug Report/Automation Exercise Defect Log.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug Report" sheetId="1" r:id="R174034ccae5e48c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="2" r:id="R4c92fa76c31442ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug Report" sheetId="1" r:id="Red2ee93dd8054d92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="2" r:id="R6d0e55783d8d4c52"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -12,9 +12,6 @@
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
     <x:t xml:space="preserve">Automation Exercise Defect Reports</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Project: Automation Exercise Ecommerce Website QA Testing | Record one independently reproducible defect per row</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Total Defects</x:t>
@@ -1490,8 +1487,8 @@
       <x:c r="U1" s="11"/>
     </x:row>
     <x:row r="2" ht="23" customHeight="1">
-      <x:c r="A2" s="12" t="s">
-        <x:v>1</x:v>
+      <x:c r="A2" s="12" t="str">
+        <x:v>Project: Automation Exercise Ecommerce Website QA Testing | Six Jira defects reconciled through 2026-08-21 | Record one independently reproducible defect per row</x:v>
       </x:c>
       <x:c r="B2" s="12"/>
       <x:c r="C2" s="12"/>
@@ -1516,7 +1513,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="13" t="s">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B4" s="14"/>
       <x:c r="D4" s="13" t="str">
@@ -1524,15 +1521,15 @@
       </x:c>
       <x:c r="E4" s="14"/>
       <x:c r="G4" s="13" t="s">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H4" s="14"/>
       <x:c r="J4" s="13" t="s">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K4" s="14"/>
       <x:c r="M4" s="17" t="s">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N4" s="18"/>
       <x:c r="O4" s="18"/>
@@ -1579,280 +1576,280 @@
     </x:row>
     <x:row r="7" ht="40" customHeight="1">
       <x:c r="A7" s="23" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B7" s="24" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B7" s="24" t="s">
+      <x:c r="C7" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="C7" s="24" t="s">
+      <x:c r="D7" s="24" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="D7" s="24" t="s">
+      <x:c r="E7" s="24" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="E7" s="24" t="s">
+      <x:c r="F7" s="24" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="F7" s="24" t="s">
+      <x:c r="G7" s="24" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="G7" s="24" t="s">
+      <x:c r="H7" s="24" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="H7" s="24" t="s">
+      <x:c r="I7" s="24" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="I7" s="24" t="s">
+      <x:c r="J7" s="24" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="J7" s="24" t="s">
+      <x:c r="K7" s="24" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="K7" s="24" t="s">
+      <x:c r="L7" s="24" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="L7" s="24" t="s">
+      <x:c r="M7" s="24" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="M7" s="24" t="s">
+      <x:c r="N7" s="24" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="N7" s="24" t="s">
+      <x:c r="O7" s="24" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="O7" s="24" t="s">
+      <x:c r="P7" s="24" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="P7" s="24" t="s">
+      <x:c r="Q7" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="Q7" s="24" t="s">
+      <x:c r="R7" s="24" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="R7" s="24" t="s">
+      <x:c r="S7" s="24" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="S7" s="24" t="s">
+      <x:c r="T7" s="24" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="T7" s="24" t="s">
+      <x:c r="U7" s="25" t="s">
         <x:v>25</x:v>
-      </x:c>
-      <x:c r="U7" s="25" t="s">
-        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="190" customHeight="1">
       <x:c r="A8" s="26" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B8" s="27" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="B8" s="27" t="s">
+      <x:c r="C8" s="27" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="C8" s="27" t="s">
+      <x:c r="D8" s="27" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="D8" s="27" t="s">
+      <x:c r="E8" s="28" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="E8" s="28" t="s">
+      <x:c r="F8" s="27" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="F8" s="27" t="s">
+      <x:c r="G8" s="27" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="G8" s="27" t="s">
+      <x:c r="H8" s="28" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="H8" s="28" t="s">
+      <x:c r="I8" s="28" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="I8" s="28" t="s">
+      <x:c r="J8" s="28" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="J8" s="28" t="s">
+      <x:c r="K8" s="28" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="K8" s="28" t="s">
+      <x:c r="L8" s="28" t="s">
         <x:v>37</x:v>
-      </x:c>
-      <x:c r="L8" s="28" t="s">
-        <x:v>38</x:v>
       </x:c>
       <x:c r="M8" s="27" t="str">
         <x:v>Selected for Development</x:v>
       </x:c>
       <x:c r="N8" s="27" t="s">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="O8" s="29">
         <x:v>46232</x:v>
       </x:c>
       <x:c r="P8" s="27" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="Q8" s="27"/>
       <x:c r="R8" s="27"/>
       <x:c r="S8" s="27" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="T8" s="29"/>
       <x:c r="U8" s="30" t="s">
-        <x:v>42</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="190" customHeight="1">
       <x:c r="A9" s="26" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B9" s="27" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C9" s="27" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D9" s="27" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="B9" s="27" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C9" s="27" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D9" s="27" t="s">
+      <x:c r="E9" s="28" t="s">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="E9" s="28" t="s">
+      <x:c r="F9" s="27" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G9" s="27" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="H9" s="28" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="F9" s="27" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="G9" s="27" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="H9" s="28" t="s">
+      <x:c r="I9" s="28" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="J9" s="28" t="s">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="I9" s="28" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="J9" s="28" t="s">
+      <x:c r="K9" s="28" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="K9" s="28" t="s">
+      <x:c r="L9" s="28" t="s">
         <x:v>48</x:v>
-      </x:c>
-      <x:c r="L9" s="28" t="s">
-        <x:v>49</x:v>
       </x:c>
       <x:c r="M9" s="27" t="str">
         <x:v>Selected for Development</x:v>
       </x:c>
       <x:c r="N9" s="27" t="s">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="O9" s="29">
         <x:v>46232</x:v>
       </x:c>
       <x:c r="P9" s="27" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="Q9" s="27"/>
       <x:c r="R9" s="27"/>
       <x:c r="S9" s="27" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="T9" s="29"/>
       <x:c r="U9" s="30" t="s">
-        <x:v>50</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="190" customHeight="1">
       <x:c r="A10" s="26" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B10" s="27" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="B10" s="27" t="s">
+      <x:c r="C10" s="27" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="C10" s="27" t="s">
+      <x:c r="D10" s="27" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="D10" s="27" t="s">
+      <x:c r="E10" s="28" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="E10" s="28" t="s">
+      <x:c r="F10" s="27" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="G10" s="27" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="H10" s="28" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="F10" s="27" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="G10" s="27" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="H10" s="28" t="s">
+      <x:c r="I10" s="28" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="I10" s="28" t="s">
+      <x:c r="J10" s="28" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="J10" s="28" t="s">
+      <x:c r="K10" s="28" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="K10" s="28" t="s">
+      <x:c r="L10" s="28" t="s">
         <x:v>59</x:v>
-      </x:c>
-      <x:c r="L10" s="28" t="s">
-        <x:v>60</x:v>
       </x:c>
       <x:c r="M10" s="27" t="str">
         <x:v>Selected for Development</x:v>
       </x:c>
       <x:c r="N10" s="27" t="s">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="O10" s="29">
         <x:v>46233</x:v>
       </x:c>
       <x:c r="P10" s="27" t="s">
-        <x:v>61</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="Q10" s="27"/>
       <x:c r="R10" s="27"/>
       <x:c r="S10" s="27" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="T10" s="29"/>
       <x:c r="U10" s="30"/>
     </x:row>
     <x:row r="11" ht="190" customHeight="1">
       <x:c r="A11" s="26" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="B11" s="27" t="s">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="B11" s="27" t="s">
+      <x:c r="C11" s="27" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="D11" s="27" t="s">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="C11" s="27" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="D11" s="27" t="s">
+      <x:c r="E11" s="28" t="s">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="E11" s="28" t="s">
+      <x:c r="F11" s="27" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G11" s="27" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="H11" s="28" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="I11" s="28" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="J11" s="28" t="s">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="F11" s="27" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="G11" s="27" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="H11" s="28" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="I11" s="28" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="J11" s="28" t="s">
+      <x:c r="K11" s="28" t="s">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="K11" s="28" t="s">
+      <x:c r="L11" s="28" t="s">
         <x:v>67</x:v>
-      </x:c>
-      <x:c r="L11" s="28" t="s">
-        <x:v>68</x:v>
       </x:c>
       <x:c r="M11" s="27" t="str">
         <x:v>Done</x:v>
@@ -1884,46 +1881,46 @@
     </x:row>
     <x:row r="12" ht="72" customHeight="1">
       <x:c r="A12" s="26" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="B12" s="27" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="B12" s="27" t="s">
+      <x:c r="C12" s="27" t="s">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="C12" s="27" t="s">
+      <x:c r="D12" s="27" t="s">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="D12" s="27" t="s">
+      <x:c r="E12" s="28" t="s">
         <x:v>72</x:v>
       </x:c>
-      <x:c r="E12" s="28" t="s">
+      <x:c r="F12" s="27" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="G12" s="27" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="H12" s="28" t="s">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="F12" s="27" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="G12" s="27" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="H12" s="28" t="s">
+      <x:c r="I12" s="28" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="I12" s="28" t="s">
+      <x:c r="J12" s="28" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="J12" s="28" t="s">
+      <x:c r="K12" s="28" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="K12" s="28" t="s">
+      <x:c r="L12" s="28" t="s">
         <x:v>77</x:v>
-      </x:c>
-      <x:c r="L12" s="28" t="s">
-        <x:v>78</x:v>
       </x:c>
       <x:c r="M12" s="27" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="N12" s="27" t="s">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="O12" s="29">
         <x:v>46235.666666666664</x:v>
@@ -1952,46 +1949,46 @@
     </x:row>
     <x:row r="13" ht="72" customHeight="1">
       <x:c r="A13" s="31" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="B13" s="32" t="s">
         <x:v>79</x:v>
       </x:c>
-      <x:c r="B13" s="32" t="s">
+      <x:c r="C13" s="32" t="s">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="C13" s="32" t="s">
+      <x:c r="D13" s="32" t="s">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="D13" s="32" t="s">
+      <x:c r="E13" s="33" t="s">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="E13" s="33" t="s">
+      <x:c r="F13" s="32" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G13" s="32" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="H13" s="33" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="F13" s="32" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="G13" s="32" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="H13" s="33" t="s">
+      <x:c r="I13" s="33" t="s">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="I13" s="33" t="s">
+      <x:c r="J13" s="33" t="s">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="J13" s="33" t="s">
+      <x:c r="K13" s="33" t="s">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="K13" s="33" t="s">
+      <x:c r="L13" s="33" t="s">
         <x:v>87</x:v>
-      </x:c>
-      <x:c r="L13" s="33" t="s">
-        <x:v>88</x:v>
       </x:c>
       <x:c r="M13" s="32" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="N13" s="32" t="s">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="O13" s="34">
         <x:v>46235.666666666664</x:v>
@@ -2425,7 +2422,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1ecf80d5678441c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cfab66c50274372"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2443,147 +2440,147 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="8" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="B1" s="9" t="s">
         <x:v>89</x:v>
       </x:c>
-      <x:c r="B1" s="9" t="s">
+      <x:c r="C1" s="9" t="s">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="C1" s="9" t="s">
-        <x:v>91</x:v>
-      </x:c>
       <x:c r="D1" s="9" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="E1" s="10" t="s">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="B2" s="1" t="s">
+      <x:c r="C2" s="1" t="s">
         <x:v>93</x:v>
-      </x:c>
-      <x:c r="C2" s="1" t="s">
-        <x:v>94</x:v>
       </x:c>
       <x:c r="D2" s="1" t="str">
         <x:v>Selected for Development</x:v>
       </x:c>
       <x:c r="E2" s="4" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="B3" s="1" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="B3" s="1" t="s">
-        <x:v>96</x:v>
-      </x:c>
       <x:c r="C3" s="1" t="s">
-        <x:v>33</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D3" s="1" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E3" s="4" t="s">
-        <x:v>97</x:v>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="3" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B4" s="1" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B4" s="1" t="s">
-        <x:v>30</x:v>
-      </x:c>
       <x:c r="C4" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D4" s="1" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="E4" s="4" t="s">
         <x:v>98</x:v>
-      </x:c>
-      <x:c r="E4" s="4" t="s">
-        <x:v>99</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="3" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B5" s="1" t="s">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="C5" s="1" t="s">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="C5" s="1" t="s">
+      <x:c r="D5" s="1" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E5" s="4" t="s">
         <x:v>101</x:v>
-      </x:c>
-      <x:c r="D5" s="1" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="E5" s="4" t="s">
-        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="3" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B6" s="1" t="s">
         <x:v>103</x:v>
-      </x:c>
-      <x:c r="B6" s="1" t="s">
-        <x:v>104</x:v>
       </x:c>
       <x:c r="C6" s="1"/>
       <x:c r="D6" s="1" t="s">
-        <x:v>105</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="E6" s="4"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="3" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B7" s="1" t="s">
-        <x:v>106</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="C7" s="1"/>
       <x:c r="D7" s="1" t="s">
-        <x:v>107</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="E7" s="4"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="3" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="B8" s="1" t="s">
         <x:v>108</x:v>
-      </x:c>
-      <x:c r="B8" s="1" t="s">
-        <x:v>109</x:v>
       </x:c>
       <x:c r="C8" s="1"/>
       <x:c r="D8" s="1" t="s">
-        <x:v>110</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="E8" s="4"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="3" t="s">
-        <x:v>81</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="B9" s="1" t="s">
-        <x:v>111</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C9" s="1"/>
       <x:c r="D9" s="1" t="s">
-        <x:v>112</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="E9" s="4"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="3" t="s">
-        <x:v>113</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B10" s="1" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C10" s="1"/>
       <x:c r="D10" s="1"/>
@@ -2591,10 +2588,10 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="3" t="s">
-        <x:v>114</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="B11" s="1" t="s">
-        <x:v>64</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C11" s="1"/>
       <x:c r="D11" s="1"/>
@@ -2603,7 +2600,7 @@
     <x:row r="12">
       <x:c r="A12" s="3"/>
       <x:c r="B12" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C12" s="1"/>
       <x:c r="D12" s="1"/>
@@ -2612,7 +2609,7 @@
     <x:row r="13">
       <x:c r="A13" s="5"/>
       <x:c r="B13" s="6" t="s">
-        <x:v>82</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C13" s="6"/>
       <x:c r="D13" s="6"/>

</xml_diff>